<commit_message>
docs: complete production planning nonlinear tutorial
- Write full RST content for the nonlinear tutorial (problem statement,
  summary of changes, conceptual model definition, setup files)
- Add structure_variables.yml material file for the tutorial
- Fix notebook title and description; call run_model with integrated_problems=True
- Downloadable material prepared.
</commit_message>
<xml_diff>
--- a/docs/source/tutorials/production_planning_nonlinear/materials/concept.xlsx
+++ b/docs/source/tutorials/production_planning_nonlinear/materials/concept.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git_repos\pyesm\tests\models\integrated\1_coupled_model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\cvxlab\docs\source\tutorials\production_planning_nonlinear\materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585653E9-AD79-4524-93C3-E1C0C5A85BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC5468E-7C6E-4C1A-B4CC-659F5F66A88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38490" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="1" sheetId="1" r:id="rId1"/>
-    <sheet name="2" sheetId="2" r:id="rId2"/>
+    <sheet name="production" sheetId="1" r:id="rId1"/>
+    <sheet name="profit" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="OpenSolver_ChosenSolver" localSheetId="0" hidden="1">Gurobi</definedName>
+    <definedName name="OpenSolver_ChosenSolver" localSheetId="0" hidden="1">CBC</definedName>
     <definedName name="OpenSolver_ChosenSolver" localSheetId="1" hidden="1">CBC</definedName>
     <definedName name="OpenSolver_DualsNewSheet" localSheetId="0" hidden="1">0</definedName>
     <definedName name="OpenSolver_DualsNewSheet" localSheetId="1" hidden="1">0</definedName>
@@ -25,8 +25,8 @@
     <definedName name="OpenSolver_LinearityCheck" localSheetId="1" hidden="1">1</definedName>
     <definedName name="OpenSolver_UpdateSensitivity" localSheetId="0" hidden="1">1</definedName>
     <definedName name="OpenSolver_UpdateSensitivity" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_adj" localSheetId="0" hidden="1">'1'!$E$4:$F$4</definedName>
-    <definedName name="solver_adj" localSheetId="1" hidden="1">'2'!$E$4:$F$4</definedName>
+    <definedName name="solver_adj" localSheetId="0" hidden="1">production!$E$4:$F$4</definedName>
+    <definedName name="solver_adj" localSheetId="1" hidden="1">profit!$E$4:$F$4</definedName>
     <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
@@ -35,26 +35,32 @@
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">'1'!$D$11</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">'2'!$E$11:$F$11</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">'1'!$E$4:$F$4</definedName>
-    <definedName name="solver_lhs3" localSheetId="0" hidden="1">'1'!$F$3</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">production!$D$13</definedName>
+    <definedName name="solver_lhs1" localSheetId="1" hidden="1">profit!$E$10:$F$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">production!$D$14</definedName>
+    <definedName name="solver_lhs2" localSheetId="1" hidden="1">profit!#REF!</definedName>
+    <definedName name="solver_lhs3" localSheetId="0" hidden="1">production!$E$4:$F$4</definedName>
+    <definedName name="solver_lhs3" localSheetId="1" hidden="1">profit!$E$5:$F$5</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="0" hidden="1">'1'!$D$10</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">'2'!$D$10</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">production!$D$12</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">profit!$E$7</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_rhs1" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_rhs3" localSheetId="0" hidden="1">'1'!$H$3</definedName>
+    <definedName name="solver_rhs2" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_rhs3" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_rhs3" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
@@ -66,7 +72,7 @@
     <definedName name="solver_tol" localSheetId="0" hidden="1">0.05</definedName>
     <definedName name="solver_tol" localSheetId="1" hidden="1">0.05</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
   </definedNames>
@@ -90,21 +96,34 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="41">
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
   <si>
     <t>u</t>
   </si>
   <si>
-    <t>Problem 1 - production optimization with variable costs</t>
-  </si>
-  <si>
     <t>prod 1</t>
   </si>
   <si>
@@ -129,9 +148,6 @@
     <t>type</t>
   </si>
   <si>
-    <t>endogenous</t>
-  </si>
-  <si>
     <t>unit profit</t>
   </si>
   <si>
@@ -162,9 +178,6 @@
     <t>total</t>
   </si>
   <si>
-    <t>J/u</t>
-  </si>
-  <si>
     <t>positive production</t>
   </si>
   <si>
@@ -180,49 +193,84 @@
     <t>energy availability</t>
   </si>
   <si>
-    <t>Problem 2 - energy use depending on production volumes</t>
-  </si>
-  <si>
-    <t>Z==1</t>
-  </si>
-  <si>
-    <t>unit energy cons initial</t>
-  </si>
-  <si>
-    <t>a_0</t>
-  </si>
-  <si>
-    <t>learning rate</t>
-  </si>
-  <si>
-    <t>lr</t>
-  </si>
-  <si>
-    <t>a-lr*x-a_0==0</t>
-  </si>
-  <si>
-    <t>from 1 to 2</t>
-  </si>
-  <si>
-    <t>from 2 to 1</t>
-  </si>
-  <si>
-    <t>a*x-b&lt;=0</t>
-  </si>
-  <si>
-    <t>a1</t>
-  </si>
-  <si>
-    <t>a2</t>
+    <t>Production optimization with fixed costs</t>
+  </si>
+  <si>
+    <t>kWh/u</t>
+  </si>
+  <si>
+    <t>unit material use</t>
+  </si>
+  <si>
+    <t>material availability</t>
+  </si>
+  <si>
+    <t>kWh</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>kg/u</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>e*x-E&lt;=0</t>
+  </si>
+  <si>
+    <t>m*x-M&lt;=0</t>
+  </si>
+  <si>
+    <t>unit profit initial</t>
+  </si>
+  <si>
+    <t>economy of scale</t>
+  </si>
+  <si>
+    <t>hybrid</t>
+  </si>
+  <si>
+    <t>c_0</t>
+  </si>
+  <si>
+    <t>change in unit profit</t>
+  </si>
+  <si>
+    <t>c1</t>
+  </si>
+  <si>
+    <t>c2</t>
+  </si>
+  <si>
+    <t>problem 1: endogenous; problem 2: exogenous</t>
+  </si>
+  <si>
+    <t>problem 1: exogenous; problem 2: endogenous</t>
+  </si>
+  <si>
+    <t>c_s</t>
+  </si>
+  <si>
+    <t>c - c_s*x - c_0 == 0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -283,11 +331,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -308,7 +358,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -340,17 +390,17 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'2'!$E$15</c:f>
+              <c:f>profit!$J$15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>a1</c:v>
+                  <c:v>c1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
+            <a:ln w="25400" cap="rnd">
               <a:noFill/>
               <a:round/>
             </a:ln>
@@ -401,8 +451,8 @@
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-0.16795428696412948"/>
-                  <c:y val="-5.927384076990376E-4"/>
+                  <c:x val="-1.3430012334873615E-2"/>
+                  <c:y val="-3.8717268848453973E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
@@ -434,120 +484,60 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'2'!$D$16:$D$33</c:f>
+              <c:f>profit!$I$16:$I$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>25</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>35</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>55</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>65</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>70</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>75</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>80</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'2'!$E$16:$E$33</c:f>
+              <c:f>profit!$J$16:$J$22</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>0.9</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.86</c:v>
+                  <c:v>1.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.82000000000000006</c:v>
+                  <c:v>1.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.78</c:v>
+                  <c:v>1.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.74</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.7</c:v>
+                  <c:v>2.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.66</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.62</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.58000000000000007</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.54</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.46</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.42000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.38</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.33999999999999997</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.30000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.26</c:v>
+                  <c:v>2.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -555,7 +545,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8E35-4D72-BAAC-EA6A31B8C468}"/>
+              <c16:uniqueId val="{00000002-CB40-43D4-8D69-5A28455E3598}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -564,17 +554,17 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'2'!$F$15</c:f>
+              <c:f>profit!$K$15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>a2</c:v>
+                  <c:v>c2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
+            <a:ln w="25400" cap="rnd">
               <a:noFill/>
               <a:round/>
             </a:ln>
@@ -625,8 +615,8 @@
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-2.6287620297462816E-2"/>
-                  <c:y val="4.9049285505978417E-2"/>
+                  <c:x val="0.11902546246067379"/>
+                  <c:y val="7.9595387100322462E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
@@ -658,120 +648,60 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'2'!$D$16:$D$33</c:f>
+              <c:f>profit!$I$16:$I$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>25</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>35</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>55</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>65</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>70</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>75</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>80</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'2'!$F$16:$F$33</c:f>
+              <c:f>profit!$K$16:$K$22</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>1.2</c:v>
+                  <c:v>2.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.19</c:v>
+                  <c:v>2.7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.18</c:v>
+                  <c:v>3.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.17</c:v>
+                  <c:v>3.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1599999999999999</c:v>
+                  <c:v>4.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.1499999999999999</c:v>
+                  <c:v>4.7</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.1399999999999999</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.1299999999999999</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.1199999999999999</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.1099999999999999</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.0999999999999999</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.0899999999999999</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.08</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.0699999999999998</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.06</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>1.05</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>1.04</c:v>
+                  <c:v>5.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -779,7 +709,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8E35-4D72-BAAC-EA6A31B8C468}"/>
+              <c16:uniqueId val="{00000005-CB40-43D4-8D69-5A28455E3598}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -798,7 +728,6 @@
         <c:axId val="1789802592"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="80"/>
           <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -942,7 +871,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="it-IT" sz="1050"/>
-                  <a:t>Unit energy use [J/u]</a:t>
+                  <a:t>Unit profit [€/u]</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1084,6 +1013,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1091,7 +1021,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1685,27 +1614,29 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>156307</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>101112</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>213353</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>43519</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>19538</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>60082</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>72311</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>48281</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="10" name="Chart 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0087FA2F-2C3B-112F-B0B9-8BD4E743AFD0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1224763-09EE-4DF5-A3A2-66530921FFE4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -1985,7 +1916,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.6328125" customWidth="1"/>
@@ -1993,164 +1925,218 @@
     <col min="3" max="4" width="7.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>176.47058999999999</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="E5" s="7">
+        <v>1.8823529999999999</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="J5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1.7</v>
+      </c>
+      <c r="F6" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5">
-        <v>3</v>
-      </c>
-      <c r="F4" s="5">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="5">
+        <f t="array" ref="D12">MMULT(E4:F4,TRANSPOSE(E5:F5))</f>
+        <v>332.17994449826995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="6">
+        <f t="array" ref="D13">MMULT(E6:F6,TRANSPOSE(E4:F4))-G8</f>
+        <v>2.9999999924257281E-6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="6" cm="1">
+        <f t="array" ref="D14">MMULT(E7:F7,TRANSPOSE(E4:F4))-G9</f>
+        <v>-1.7647050000000064</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
         <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="8">
-        <v>1</v>
-      </c>
-      <c r="F5" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="6">
-        <v>5</v>
-      </c>
-      <c r="F6" s="6">
-        <v>10</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10">
-        <f t="array" ref="D10">MMULT(E4:F4,TRANSPOSE(E5:F5))</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="3">
-        <f t="array" ref="D11">MMULT(E6:F6,TRANSPOSE(E4:F4))-G7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2161,8 +2147,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1A5120-BA3A-4F72-9BE3-44BB5F6207EF}">
-  <dimension ref="A1:H33"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD001682-046D-428E-BCD5-8AEA5ED73DC2}">
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.6328125" customWidth="1"/>
@@ -2170,376 +2156,245 @@
     <col min="3" max="4" width="7.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="E4" s="4">
+        <v>1.8823529999999999</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7">
+        <v>176.47058999999999</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F7">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="3" cm="1">
+        <f t="array" ref="E10:F10">E4:F4-E6:F6-E7:F7*E5:F5</f>
+        <v>5.0000000029193359E-8</v>
+      </c>
+      <c r="F10" s="3">
         <v>0</v>
       </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0.9</v>
-      </c>
-      <c r="F4" s="4">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="H4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I15" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" cm="1">
+        <f t="array" ref="J16:K16">$E$6:$F$6+$E$7:$F$7*I16</f>
+        <v>1</v>
+      </c>
+      <c r="K16" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I17">
+        <v>50</v>
+      </c>
+      <c r="J17" s="3" cm="1">
+        <f t="array" ref="J17:K17">$E$6:$F$6+$E$7:$F$7*I17</f>
+        <v>1.25</v>
+      </c>
+      <c r="K17" s="3">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="18" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I18">
+        <v>100</v>
+      </c>
+      <c r="J18" s="3" cm="1">
+        <f t="array" ref="J18:K18">$E$6:$F$6+$E$7:$F$7*I18</f>
+        <v>1.5</v>
+      </c>
+      <c r="K18" s="3">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="19" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I19">
+        <v>150</v>
+      </c>
+      <c r="J19" s="3" cm="1">
+        <f t="array" ref="J19:K19">$E$6:$F$6+$E$7:$F$7*I19</f>
+        <v>1.75</v>
+      </c>
+      <c r="K19" s="3">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="20" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I20">
+        <v>200</v>
+      </c>
+      <c r="J20" s="3" cm="1">
+        <f t="array" ref="J20:K20">$E$6:$F$6+$E$7:$F$7*I20</f>
         <v>2</v>
       </c>
-      <c r="E5" s="7">
-        <v>0</v>
-      </c>
-      <c r="F5" s="7">
-        <v>20</v>
-      </c>
-      <c r="H5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0.9</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7">
-        <v>-8.0000000000000002E-3</v>
-      </c>
-      <c r="F7">
-        <v>-2E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3">
-        <f t="array" ref="E11:F11">E4:F4-E6:F6-E7:F7*E5:F5</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3">
-        <f t="array" ref="E16:F16">$E$6:$F$6+$E$7:$F$7*D16</f>
-        <v>0.9</v>
-      </c>
-      <c r="F16" s="3">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="17" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D17">
-        <v>5</v>
-      </c>
-      <c r="E17" s="3">
-        <f t="array" ref="E17:F17">$E$6:$F$6+$E$7:$F$7*D17</f>
-        <v>0.86</v>
-      </c>
-      <c r="F17" s="3">
-        <v>1.19</v>
-      </c>
-    </row>
-    <row r="18" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D18">
-        <v>10</v>
-      </c>
-      <c r="E18" s="3">
-        <f t="array" ref="E18:F18">$E$6:$F$6+$E$7:$F$7*D18</f>
-        <v>0.82000000000000006</v>
-      </c>
-      <c r="F18" s="3">
-        <v>1.18</v>
-      </c>
-    </row>
-    <row r="19" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D19">
-        <v>15</v>
-      </c>
-      <c r="E19" s="3">
-        <f t="array" ref="E19:F19">$E$6:$F$6+$E$7:$F$7*D19</f>
-        <v>0.78</v>
-      </c>
-      <c r="F19" s="3">
-        <v>1.17</v>
-      </c>
-    </row>
-    <row r="20" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D20">
-        <v>20</v>
-      </c>
-      <c r="E20" s="3">
-        <f t="array" ref="E20:F20">$E$6:$F$6+$E$7:$F$7*D20</f>
-        <v>0.74</v>
-      </c>
-      <c r="F20" s="3">
-        <v>1.1599999999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D21">
-        <v>25</v>
-      </c>
-      <c r="E21" s="3">
-        <f t="array" ref="E21:F21">$E$6:$F$6+$E$7:$F$7*D21</f>
-        <v>0.7</v>
-      </c>
-      <c r="F21" s="3">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="22" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D22">
-        <v>30</v>
-      </c>
-      <c r="E22" s="3">
-        <f t="array" ref="E22:F22">$E$6:$F$6+$E$7:$F$7*D22</f>
-        <v>0.66</v>
-      </c>
-      <c r="F22" s="3">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="23" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D23">
-        <v>35</v>
-      </c>
-      <c r="E23" s="3">
-        <f t="array" ref="E23:F23">$E$6:$F$6+$E$7:$F$7*D23</f>
-        <v>0.62</v>
-      </c>
-      <c r="F23" s="3">
-        <v>1.1299999999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D24">
-        <v>40</v>
-      </c>
-      <c r="E24" s="3">
-        <f t="array" ref="E24:F24">$E$6:$F$6+$E$7:$F$7*D24</f>
-        <v>0.58000000000000007</v>
-      </c>
-      <c r="F24" s="3">
-        <v>1.1199999999999999</v>
-      </c>
-    </row>
-    <row r="25" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D25">
-        <v>45</v>
-      </c>
-      <c r="E25" s="3">
-        <f t="array" ref="E25:F25">$E$6:$F$6+$E$7:$F$7*D25</f>
-        <v>0.54</v>
-      </c>
-      <c r="F25" s="3">
-        <v>1.1099999999999999</v>
-      </c>
-    </row>
-    <row r="26" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D26">
-        <v>50</v>
-      </c>
-      <c r="E26" s="3">
-        <f t="array" ref="E26:F26">$E$6:$F$6+$E$7:$F$7*D26</f>
-        <v>0.5</v>
-      </c>
-      <c r="F26" s="3">
-        <v>1.0999999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D27">
-        <v>55</v>
-      </c>
-      <c r="E27" s="3">
-        <f t="array" ref="E27:F27">$E$6:$F$6+$E$7:$F$7*D27</f>
-        <v>0.46</v>
-      </c>
-      <c r="F27" s="3">
-        <v>1.0899999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D28">
-        <v>60</v>
-      </c>
-      <c r="E28" s="3">
-        <f t="array" ref="E28:F28">$E$6:$F$6+$E$7:$F$7*D28</f>
-        <v>0.42000000000000004</v>
-      </c>
-      <c r="F28" s="3">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="29" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D29">
-        <v>65</v>
-      </c>
-      <c r="E29" s="3">
-        <f t="array" ref="E29:F29">$E$6:$F$6+$E$7:$F$7*D29</f>
-        <v>0.38</v>
-      </c>
-      <c r="F29" s="3">
-        <v>1.0699999999999998</v>
-      </c>
-    </row>
-    <row r="30" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D30">
-        <v>70</v>
-      </c>
-      <c r="E30" s="3">
-        <f t="array" ref="E30:F30">$E$6:$F$6+$E$7:$F$7*D30</f>
-        <v>0.33999999999999997</v>
-      </c>
-      <c r="F30" s="3">
-        <v>1.06</v>
-      </c>
-    </row>
-    <row r="31" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D31">
-        <v>75</v>
-      </c>
-      <c r="E31" s="3">
-        <f t="array" ref="E31:F31">$E$6:$F$6+$E$7:$F$7*D31</f>
-        <v>0.30000000000000004</v>
-      </c>
-      <c r="F31" s="3">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="32" spans="4:6" x14ac:dyDescent="0.35">
-      <c r="D32">
-        <v>80</v>
-      </c>
-      <c r="E32" s="3">
-        <f t="array" ref="E32:F32">$E$6:$F$6+$E$7:$F$7*D32</f>
-        <v>0.26</v>
-      </c>
-      <c r="F32" s="3">
-        <v>1.04</v>
-      </c>
-    </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
+      <c r="K20" s="3">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="21" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I21">
+        <v>250</v>
+      </c>
+      <c r="J21" s="3" cm="1">
+        <f t="array" ref="J21:K21">$E$6:$F$6+$E$7:$F$7*I21</f>
+        <v>2.25</v>
+      </c>
+      <c r="K21" s="3">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="22" spans="9:11" x14ac:dyDescent="0.35">
+      <c r="I22">
+        <v>300</v>
+      </c>
+      <c r="J22" s="3" cm="1">
+        <f t="array" ref="J22:K22">$E$6:$F$6+$E$7:$F$7*I22</f>
+        <v>2.5</v>
+      </c>
+      <c r="K22" s="3">
+        <v>5.2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>